<commit_message>
Completed component tests ct007 - ct010, completed model selection experiments
</commit_message>
<xml_diff>
--- a/assets/submission checklist.xlsx
+++ b/assets/submission checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cowse\aes-thesis\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80BB9468-C402-4277-A237-BD8F508515EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25048A86-AC92-4239-8C4D-4F374FB3DC4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="47">
   <si>
     <t>Name</t>
   </si>
@@ -642,11 +642,29 @@
       <c r="A12" t="s">
         <v>19</v>
       </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -662,83 +680,131 @@
       <c r="A16" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>

</xml_diff>

<commit_message>
Updated whisper_transcriptions to dict, updated EssayEditor for efficiency
</commit_message>
<xml_diff>
--- a/assets/submission checklist.xlsx
+++ b/assets/submission checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cowse\aes-thesis\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25048A86-AC92-4239-8C4D-4F374FB3DC4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B4A329-622D-4950-9A97-9A3C1AD16093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="47">
   <si>
     <t>Name</t>
   </si>
@@ -537,6 +537,9 @@
       <c r="C3" t="s">
         <v>16</v>
       </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -637,6 +640,15 @@
       <c r="A11" t="s">
         <v>18</v>
       </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -704,7 +716,10 @@
       <c r="A19" t="s">
         <v>26</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" t="s">
         <v>16</v>
       </c>
     </row>
@@ -731,6 +746,15 @@
       <c r="A22" t="s">
         <v>29</v>
       </c>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
@@ -776,6 +800,12 @@
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>36</v>
+      </c>
+      <c r="B27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Complete Whisper testing and evaluation, along with collection of audio samples
</commit_message>
<xml_diff>
--- a/assets/submission checklist.xlsx
+++ b/assets/submission checklist.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cowse\aes-thesis\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B4A329-622D-4950-9A97-9A3C1AD16093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B32630-591A-43D2-ABFB-C0406E86CA71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$1</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="48">
   <si>
     <t>Name</t>
   </si>
@@ -66,9 +69,6 @@
     <t>Skyla</t>
   </si>
   <si>
-    <t>Brice</t>
-  </si>
-  <si>
     <t>Nasri</t>
   </si>
   <si>
@@ -166,6 +166,12 @@
   </si>
   <si>
     <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>Katelyn Montoute</t>
+  </si>
+  <si>
+    <t>Bryce</t>
   </si>
 </sst>
 </file>
@@ -492,10 +498,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -515,414 +522,439 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" t="s">
-        <v>16</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="C17" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>7</v>
+      </c>
+      <c r="B19" t="s">
+        <v>15</v>
       </c>
       <c r="C19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>46</v>
+      </c>
+      <c r="B20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="B24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>34</v>
-      </c>
-      <c r="B25" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" t="s">
-        <v>16</v>
-      </c>
-      <c r="C26" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C27" t="s">
-        <v>16</v>
+        <v>15</v>
+      </c>
+      <c r="D27" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>28</v>
+      </c>
+      <c r="B28" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>4</v>
+      </c>
+      <c r="B29" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C30" t="s">
-        <v>16</v>
+        <v>15</v>
+      </c>
+      <c r="D30" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="B31" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="B32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C32" t="s">
-        <v>16</v>
+        <v>15</v>
+      </c>
+      <c r="D32" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>13</v>
-      </c>
-      <c r="B33" t="s">
-        <v>16</v>
-      </c>
-      <c r="C33" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C34" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B35" t="s">
-        <v>16</v>
-      </c>
-      <c r="C35" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>12</v>
-      </c>
-      <c r="B36" t="s">
-        <v>16</v>
-      </c>
-      <c r="C36" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>30</v>
+        <v>38</v>
+      </c>
+      <c r="B37" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>41</v>
+        <v>11</v>
+      </c>
+      <c r="B38" t="s">
+        <v>15</v>
+      </c>
+      <c r="C38" t="s">
+        <v>15</v>
       </c>
       <c r="G38" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>42</v>
+        <v>12</v>
+      </c>
+      <c r="B39" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>44</v>
+        <v>10</v>
+      </c>
+      <c r="B41" t="s">
+        <v>15</v>
+      </c>
+      <c r="C41" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>45</v>
+        <v>19</v>
+      </c>
+      <c r="B42" t="s">
+        <v>15</v>
+      </c>
+      <c r="C42" t="s">
+        <v>15</v>
+      </c>
+      <c r="D42" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D43">
+      <sortCondition ref="A1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>